<commit_message>
teamb: added about page and modified excel
</commit_message>
<xml_diff>
--- a/microsoft exel.xlsx
+++ b/microsoft exel.xlsx
@@ -9,12 +9,12 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>This is microsoft exel file</t>
   </si>
@@ -46,10 +46,7 @@
     <t>Urdu</t>
   </si>
   <si>
-    <t>total: 550</t>
-  </si>
-  <si>
-    <t>total: 370</t>
+    <t>TotAL</t>
   </si>
 </sst>
 </file>
@@ -463,7 +460,7 @@
         <v>100</v>
       </c>
       <c r="D6">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -477,7 +474,7 @@
         <v>75</v>
       </c>
       <c r="D7">
-        <v>60</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -495,11 +492,16 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C9" t="s">
+      <c r="B9" t="s">
         <v>10</v>
       </c>
-      <c r="D9" t="s">
-        <v>11</v>
+      <c r="C9">
+        <f>SUM(C4:C8)</f>
+        <v>450</v>
+      </c>
+      <c r="D9">
+        <f>SUM(D4:D8)</f>
+        <v>382</v>
       </c>
     </row>
   </sheetData>

</xml_diff>